<commit_message>
added yaml file and fixed pipeline issues
</commit_message>
<xml_diff>
--- a/testdata/logindata.xlsx
+++ b/testdata/logindata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pavan\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\opencartPlaywrightPythonFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2338C232-9E9F-4E2C-BA76-8CB052921956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D00883-62DE-4CE3-AD14-017D3FD1D644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16354" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{DD2D5C5F-8E6D-49C6-975C-904030A5775C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DD2D5C5F-8E6D-49C6-975C-904030A5775C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>testName</t>
   </si>
@@ -51,12 +51,6 @@
     <t>Valid login</t>
   </si>
   <si>
-    <t>pavanol@abc.com</t>
-  </si>
-  <si>
-    <t>test@123</t>
-  </si>
-  <si>
     <t>success</t>
   </si>
   <si>
@@ -70,16 +64,27 @@
   </si>
   <si>
     <t>failure</t>
+  </si>
+  <si>
+    <t>chethan8105@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -117,14 +122,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -141,9 +149,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -181,7 +189,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -287,7 +295,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -429,7 +437,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -463,31 +471,34 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1">
+        <v>12345678</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{74764DE6-7B87-43B7-9C34-DFDEDB22439E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>